<commit_message>
adds concept of lu:colour for authoritative colours
</commit_message>
<xml_diff>
--- a/classification-systems/nzlum/build/nzlum_v0.3.0.xlsx
+++ b/classification-systems/nzlum/build/nzlum_v0.3.0.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="NZLUM" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NZLUM" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +29,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="31">
     <fill>
       <patternFill/>
     </fill>
@@ -39,6 +39,146 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF5E3A98"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3F007D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7C76B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA39FCB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC9CAE3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE9E8F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCFBFD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA00019"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC77A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF9E17"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC8C69F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF122112"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF357735"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7F7F54"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA4A898"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4A4C39"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBFA798"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3B505B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBCBFE1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF815E5B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC19878"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB8C2CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD0D2DF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8ADFA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF72737E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE1CEA7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE77148"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD69B97"/>
       </patternFill>
     </fill>
   </fills>
@@ -54,12 +194,96 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -427,15 +651,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F96"/>
+  <dimension ref="A1:I96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -451,22 +678,37 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Primary colour</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Secondary code</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Secondary class</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Secondary colour</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Tertiary code</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Tertiary class</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Tertiary colour</t>
         </is>
       </c>
     </row>
@@ -481,354 +723,458 @@
           <t>Conservation and Minimal Use</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>1.1.0</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Nature conservation</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>1.1.1</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Strict nature reserve</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>#5E3A98</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n"/>
       <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
+      <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>1.1.2</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Wilderness area</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>#3F007D</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n"/>
       <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
+      <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>1.1.3</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>National Park</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>#7C76B6</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n"/>
       <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="n"/>
+      <c r="C5" s="2" t="inlineStr"/>
       <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>1.1.4</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Natural feature protection</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>#A39FCB</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n"/>
       <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
+      <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>1.1.5</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Habitat or species management area</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>#C9CAE3</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n"/>
       <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
+      <c r="C7" s="2" t="inlineStr"/>
       <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>1.1.6</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Protected landscape</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>#E9E8F2</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n"/>
       <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
+      <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>1.1.7</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Other conserved area</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>#FCFBFD</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n"/>
       <c r="B9" s="2" t="n"/>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>1.2.0</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Cultural and natural heritage</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>#A00019</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>1.2.1</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Indigenous cultural heritage</t>
         </is>
       </c>
+      <c r="I9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n"/>
       <c r="B10" s="2" t="n"/>
-      <c r="C10" s="2" t="n"/>
+      <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>1.2.2</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Cultural heritage</t>
         </is>
       </c>
+      <c r="I10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n"/>
       <c r="B11" s="2" t="n"/>
-      <c r="C11" s="2" t="n"/>
+      <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>1.2.3</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Natural heritage</t>
         </is>
       </c>
+      <c r="I11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n"/>
       <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>1.3.0</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Minimal use from relatively natural environments</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>#FFC77A</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>1.3.1</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Surface water supply</t>
         </is>
       </c>
+      <c r="I12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n"/>
       <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
+      <c r="C13" s="2" t="inlineStr"/>
       <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>1.3.2</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Ground water</t>
         </is>
       </c>
+      <c r="I13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n"/>
       <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
+      <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>1.3.3</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Grazing native vegetation</t>
         </is>
       </c>
+      <c r="I14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n"/>
       <c r="B15" s="2" t="n"/>
-      <c r="C15" s="2" t="n"/>
+      <c r="C15" s="2" t="inlineStr"/>
       <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>1.3.4</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Production from indigenous vegetation</t>
         </is>
       </c>
+      <c r="I15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n"/>
       <c r="B16" s="2" t="n"/>
-      <c r="C16" s="2" t="n"/>
+      <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>1.3.5</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Customary use</t>
         </is>
       </c>
+      <c r="I16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n"/>
       <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="n"/>
+      <c r="C17" s="2" t="inlineStr"/>
       <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>1.3.6</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Defence land</t>
+        </is>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>#FF9E17</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n"/>
       <c r="B18" s="2" t="n"/>
-      <c r="C18" s="2" t="n"/>
+      <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>1.3.7</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Environmental &amp; infrastructure protection</t>
         </is>
       </c>
+      <c r="I18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n"/>
       <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
+      <c r="C19" s="2" t="inlineStr"/>
       <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>1.3.8</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>Carbon forest</t>
         </is>
       </c>
+      <c r="I19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n"/>
       <c r="B20" s="2" t="n"/>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>1.4.0</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>Unused land and land in transition</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>#C8C69F</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>1.4.1</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>Unused land</t>
         </is>
       </c>
+      <c r="I20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n"/>
       <c r="B21" s="2" t="n"/>
-      <c r="C21" s="2" t="n"/>
+      <c r="C21" s="2" t="inlineStr"/>
       <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>1.4.2</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>Land undergoing rehabilitation</t>
         </is>
       </c>
+      <c r="I21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -841,562 +1187,687 @@
           <t>Production agriculture and plantations</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>2.1.0</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>Plantation forests</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="F22" s="14" t="inlineStr">
+        <is>
+          <t>#122112</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>2.1.1</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>Exotic plantation forestry</t>
         </is>
       </c>
+      <c r="I22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n"/>
       <c r="B23" s="2" t="n"/>
-      <c r="C23" s="2" t="n"/>
+      <c r="C23" s="2" t="inlineStr"/>
       <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>2.1.2</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Indigenous plantation forestry</t>
         </is>
       </c>
+      <c r="I23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n"/>
       <c r="B24" s="2" t="n"/>
-      <c r="C24" s="2" t="n"/>
+      <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>2.1.3</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Other production uses</t>
         </is>
       </c>
+      <c r="I24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n"/>
       <c r="B25" s="2" t="n"/>
-      <c r="C25" s="2" t="n"/>
+      <c r="C25" s="2" t="inlineStr"/>
       <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>2.1.4</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>Planted environmental &amp; infrastructure protection</t>
         </is>
       </c>
+      <c r="I25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n"/>
       <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
+      <c r="C26" s="2" t="inlineStr"/>
       <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>2.1.5</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>Permanent carbon forest</t>
         </is>
       </c>
+      <c r="I26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n"/>
       <c r="B27" s="2" t="n"/>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr"/>
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>2.2.0</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>Grazing modified pasture systems</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="F27" s="15" t="inlineStr">
+        <is>
+          <t>#357735</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>2.2.1</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>Dairy</t>
         </is>
       </c>
+      <c r="I27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n"/>
       <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
+      <c r="C28" s="2" t="inlineStr"/>
       <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>2.2.2</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Intensive dry stock</t>
         </is>
       </c>
+      <c r="I28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n"/>
       <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
+      <c r="C29" s="2" t="inlineStr"/>
       <c r="D29" s="2" t="n"/>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>2.2.3</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>Extensive dry stock</t>
         </is>
       </c>
+      <c r="I29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n"/>
       <c r="B30" s="2" t="n"/>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>2.3.0</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>Short-rotation and seasonal cropping</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="F30" s="16" t="inlineStr">
+        <is>
+          <t>#7F7F54</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>2.3.1</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Arable cropping</t>
         </is>
       </c>
+      <c r="I30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n"/>
       <c r="B31" s="2" t="n"/>
-      <c r="C31" s="2" t="n"/>
+      <c r="C31" s="2" t="inlineStr"/>
       <c r="D31" s="2" t="n"/>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>2.3.2</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>Arable and mixed livestock cropping</t>
         </is>
       </c>
+      <c r="I31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n"/>
       <c r="B32" s="2" t="n"/>
-      <c r="C32" s="2" t="n"/>
+      <c r="C32" s="2" t="inlineStr"/>
       <c r="D32" s="2" t="n"/>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>2.3.3</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>Short-rotation horticulture</t>
         </is>
       </c>
+      <c r="I32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n"/>
       <c r="B33" s="2" t="n"/>
-      <c r="C33" s="2" t="n"/>
+      <c r="C33" s="2" t="inlineStr"/>
       <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>2.3.4</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>Seasonal flowers and bulbs, and turf farming</t>
         </is>
       </c>
+      <c r="I33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n"/>
       <c r="B34" s="2" t="n"/>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>2.4.0</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>Perennial horticulture</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="F34" s="17" t="inlineStr">
+        <is>
+          <t>#A4A898</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>2.4.1</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>Tree crops</t>
         </is>
       </c>
+      <c r="I34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n"/>
       <c r="B35" s="2" t="n"/>
-      <c r="C35" s="2" t="n"/>
+      <c r="C35" s="2" t="inlineStr"/>
       <c r="D35" s="2" t="n"/>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>2.4.2</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>Vine fruits</t>
         </is>
       </c>
+      <c r="I35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n"/>
       <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="n"/>
+      <c r="C36" s="2" t="inlineStr"/>
       <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>2.4.3</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>Other perennial horticulture</t>
         </is>
       </c>
+      <c r="I36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n"/>
       <c r="B37" s="2" t="n"/>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr"/>
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>2.5.0</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>Intensive horticulture</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="F37" s="18" t="inlineStr">
+        <is>
+          <t>#4A4C39</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>2.5.1</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>Production nurseries</t>
         </is>
       </c>
+      <c r="I37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n"/>
       <c r="B38" s="2" t="n"/>
-      <c r="C38" s="2" t="n"/>
+      <c r="C38" s="2" t="inlineStr"/>
       <c r="D38" s="2" t="n"/>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>2.5.2</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>Glasshouses/shadehouses</t>
         </is>
       </c>
+      <c r="I38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n"/>
       <c r="B39" s="2" t="n"/>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr"/>
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>2.6.0</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>Intensive animal production</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="F39" s="19" t="inlineStr">
+        <is>
+          <t>#BFA798</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>2.6.1</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>Intensive animal containment</t>
         </is>
       </c>
+      <c r="I39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n"/>
       <c r="B40" s="2" t="n"/>
-      <c r="C40" s="2" t="n"/>
+      <c r="C40" s="2" t="inlineStr"/>
       <c r="D40" s="2" t="n"/>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>2.6.2</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>Poultry farms</t>
         </is>
       </c>
+      <c r="I40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n"/>
       <c r="B41" s="2" t="n"/>
-      <c r="C41" s="2" t="n"/>
+      <c r="C41" s="2" t="inlineStr"/>
       <c r="D41" s="2" t="n"/>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>2.6.3</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>Piggeries</t>
         </is>
       </c>
+      <c r="I41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n"/>
       <c r="B42" s="2" t="n"/>
-      <c r="C42" s="2" t="n"/>
+      <c r="C42" s="2" t="inlineStr"/>
       <c r="D42" s="2" t="n"/>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="2" t="n"/>
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>2.6.4</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>Horse studs</t>
         </is>
       </c>
+      <c r="I42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n"/>
       <c r="B43" s="2" t="n"/>
-      <c r="C43" s="2" t="n"/>
+      <c r="C43" s="2" t="inlineStr"/>
       <c r="D43" s="2" t="n"/>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+      <c r="G43" s="2" t="inlineStr">
         <is>
           <t>2.6.5</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>Aquaculture</t>
         </is>
       </c>
+      <c r="I43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n"/>
       <c r="B44" s="2" t="n"/>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>2.7.0</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>Water and wastewater</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="F44" s="20" t="inlineStr">
+        <is>
+          <t>#3B505B</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>2.7.1</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>Stock water</t>
         </is>
       </c>
+      <c r="I44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n"/>
       <c r="B45" s="2" t="n"/>
-      <c r="C45" s="2" t="n"/>
+      <c r="C45" s="2" t="inlineStr"/>
       <c r="D45" s="2" t="n"/>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>2.7.2</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>Effluent pond</t>
         </is>
       </c>
+      <c r="I45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n"/>
       <c r="B46" s="2" t="n"/>
-      <c r="C46" s="2" t="n"/>
+      <c r="C46" s="2" t="inlineStr"/>
       <c r="D46" s="2" t="n"/>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>2.7.3</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>Water treatment – land application</t>
         </is>
       </c>
+      <c r="I46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n"/>
       <c r="B47" s="2" t="n"/>
-      <c r="C47" s="2" t="n"/>
+      <c r="C47" s="2" t="inlineStr"/>
       <c r="D47" s="2" t="n"/>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E47" s="2" t="n"/>
+      <c r="F47" s="2" t="n"/>
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>2.7.4</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>Water treatment – wetland</t>
         </is>
       </c>
+      <c r="I47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n"/>
       <c r="B48" s="2" t="n"/>
-      <c r="C48" s="2" t="n"/>
+      <c r="C48" s="2" t="inlineStr"/>
       <c r="D48" s="2" t="n"/>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>2.7.5</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>Irrigation reservoirs and canals</t>
         </is>
       </c>
+      <c r="I48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n"/>
       <c r="B49" s="2" t="n"/>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr"/>
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>2.8.0</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>Land in transition</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="F49" s="21" t="inlineStr">
+        <is>
+          <t>#BCBFE1</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>2.8.1</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>Unused degraded land</t>
         </is>
       </c>
+      <c r="I49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n"/>
       <c r="B50" s="2" t="n"/>
-      <c r="C50" s="2" t="n"/>
+      <c r="C50" s="2" t="inlineStr"/>
       <c r="D50" s="2" t="n"/>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="2" t="n"/>
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>2.8.2</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>No defined use</t>
         </is>
       </c>
+      <c r="I50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n"/>
       <c r="B51" s="2" t="n"/>
-      <c r="C51" s="2" t="n"/>
+      <c r="C51" s="2" t="inlineStr"/>
       <c r="D51" s="2" t="n"/>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="2" t="n"/>
+      <c r="G51" s="2" t="inlineStr">
         <is>
           <t>2.8.3</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>Land undergoing rehabilitation</t>
         </is>
       </c>
+      <c r="I51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n"/>
       <c r="B52" s="2" t="n"/>
-      <c r="C52" s="2" t="n"/>
+      <c r="C52" s="2" t="inlineStr"/>
       <c r="D52" s="2" t="n"/>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E52" s="2" t="n"/>
+      <c r="F52" s="2" t="n"/>
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>2.8.4</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t>Abandoned land</t>
         </is>
       </c>
+      <c r="I52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -1409,829 +1880,1017 @@
           <t>Built environment</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr"/>
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>3.1.0</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>Residential</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="F53" s="22" t="inlineStr">
+        <is>
+          <t>#815E5B</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
         <is>
           <t>3.1.1</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="H53" s="2" t="inlineStr">
         <is>
           <t>High-density residential</t>
         </is>
       </c>
+      <c r="I53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n"/>
       <c r="B54" s="2" t="n"/>
-      <c r="C54" s="2" t="n"/>
+      <c r="C54" s="2" t="inlineStr"/>
       <c r="D54" s="2" t="n"/>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E54" s="2" t="n"/>
+      <c r="F54" s="2" t="n"/>
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>3.1.2</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr">
         <is>
           <t>Medium-density residential</t>
         </is>
       </c>
+      <c r="I54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n"/>
       <c r="B55" s="2" t="n"/>
-      <c r="C55" s="2" t="n"/>
+      <c r="C55" s="2" t="inlineStr"/>
       <c r="D55" s="2" t="n"/>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E55" s="2" t="n"/>
+      <c r="F55" s="2" t="n"/>
+      <c r="G55" s="2" t="inlineStr">
         <is>
           <t>3.1.3</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="H55" s="2" t="inlineStr">
         <is>
           <t>Low-density residential</t>
         </is>
       </c>
+      <c r="I55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n"/>
       <c r="B56" s="2" t="n"/>
-      <c r="C56" s="2" t="n"/>
+      <c r="C56" s="2" t="inlineStr"/>
       <c r="D56" s="2" t="n"/>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E56" s="2" t="n"/>
+      <c r="F56" s="2" t="n"/>
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>3.1.4</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>Rural residential</t>
         </is>
       </c>
+      <c r="I56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n"/>
       <c r="B57" s="2" t="n"/>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr"/>
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>3.2.0</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>Public recreation and services</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="F57" s="23" t="inlineStr">
+        <is>
+          <t>#C19878</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
         <is>
           <t>3.2.1</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="H57" s="2" t="inlineStr">
         <is>
           <t>Outdoor recreation</t>
         </is>
       </c>
+      <c r="I57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n"/>
       <c r="B58" s="2" t="n"/>
-      <c r="C58" s="2" t="n"/>
+      <c r="C58" s="2" t="inlineStr"/>
       <c r="D58" s="2" t="n"/>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E58" s="2" t="n"/>
+      <c r="F58" s="2" t="n"/>
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>3.2.2</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="H58" s="2" t="inlineStr">
         <is>
           <t>Indoor recreation</t>
         </is>
       </c>
+      <c r="I58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n"/>
       <c r="B59" s="2" t="n"/>
-      <c r="C59" s="2" t="n"/>
+      <c r="C59" s="2" t="inlineStr"/>
       <c r="D59" s="2" t="n"/>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E59" s="2" t="n"/>
+      <c r="F59" s="2" t="n"/>
+      <c r="G59" s="2" t="inlineStr">
         <is>
           <t>3.2.3</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t>Community services</t>
         </is>
       </c>
+      <c r="I59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n"/>
       <c r="B60" s="2" t="n"/>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr"/>
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>3.3.0</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>Commercial</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="F60" s="24" t="inlineStr">
+        <is>
+          <t>#B8C2CE</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
         <is>
           <t>3.3.1</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>Retail</t>
         </is>
       </c>
+      <c r="I60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n"/>
       <c r="B61" s="2" t="n"/>
-      <c r="C61" s="2" t="n"/>
+      <c r="C61" s="2" t="inlineStr"/>
       <c r="D61" s="2" t="n"/>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E61" s="2" t="n"/>
+      <c r="F61" s="2" t="n"/>
+      <c r="G61" s="2" t="inlineStr">
         <is>
           <t>3.3.2</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="H61" s="2" t="inlineStr">
         <is>
           <t>Office</t>
         </is>
       </c>
+      <c r="I61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n"/>
       <c r="B62" s="2" t="n"/>
-      <c r="C62" s="2" t="n"/>
+      <c r="C62" s="2" t="inlineStr"/>
       <c r="D62" s="2" t="n"/>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="E62" s="2" t="n"/>
+      <c r="F62" s="2" t="n"/>
+      <c r="G62" s="2" t="inlineStr">
         <is>
           <t>3.3.3</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr">
+      <c r="H62" s="2" t="inlineStr">
         <is>
           <t>Hospitality</t>
         </is>
       </c>
+      <c r="I62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n"/>
       <c r="B63" s="2" t="n"/>
-      <c r="C63" s="2" t="n"/>
+      <c r="C63" s="2" t="inlineStr"/>
       <c r="D63" s="2" t="n"/>
-      <c r="E63" s="2" t="inlineStr">
+      <c r="E63" s="2" t="n"/>
+      <c r="F63" s="2" t="n"/>
+      <c r="G63" s="2" t="inlineStr">
         <is>
           <t>3.3.4</t>
         </is>
       </c>
-      <c r="F63" s="2" t="inlineStr">
+      <c r="H63" s="2" t="inlineStr">
         <is>
           <t>Entertainment</t>
         </is>
       </c>
+      <c r="I63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n"/>
       <c r="B64" s="2" t="n"/>
-      <c r="C64" s="2" t="n"/>
+      <c r="C64" s="2" t="inlineStr"/>
       <c r="D64" s="2" t="n"/>
-      <c r="E64" s="2" t="inlineStr">
+      <c r="E64" s="2" t="n"/>
+      <c r="F64" s="2" t="n"/>
+      <c r="G64" s="2" t="inlineStr">
         <is>
           <t>3.3.5</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr">
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t>Healthcare</t>
         </is>
       </c>
+      <c r="I64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n"/>
       <c r="B65" s="2" t="n"/>
-      <c r="C65" s="2" t="n"/>
+      <c r="C65" s="2" t="inlineStr"/>
       <c r="D65" s="2" t="n"/>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="E65" s="2" t="n"/>
+      <c r="F65" s="2" t="n"/>
+      <c r="G65" s="2" t="inlineStr">
         <is>
           <t>3.3.6</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="H65" s="2" t="inlineStr">
         <is>
           <t>Transportation &amp; warehousing</t>
         </is>
       </c>
+      <c r="I65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n"/>
       <c r="B66" s="2" t="n"/>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr"/>
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>3.4.0</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>Manufacturing and industrial</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="F66" s="25" t="inlineStr">
+        <is>
+          <t>#D0D2DF</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
         <is>
           <t>3.4.1</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="H66" s="2" t="inlineStr">
         <is>
           <t>General purpose factory</t>
         </is>
       </c>
+      <c r="I66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n"/>
       <c r="B67" s="2" t="n"/>
-      <c r="C67" s="2" t="n"/>
+      <c r="C67" s="2" t="inlineStr"/>
       <c r="D67" s="2" t="n"/>
-      <c r="E67" s="2" t="inlineStr">
+      <c r="E67" s="2" t="n"/>
+      <c r="F67" s="2" t="n"/>
+      <c r="G67" s="2" t="inlineStr">
         <is>
           <t>3.4.2</t>
         </is>
       </c>
-      <c r="F67" s="2" t="inlineStr">
+      <c r="H67" s="2" t="inlineStr">
         <is>
           <t>Food processing factory</t>
         </is>
       </c>
+      <c r="I67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n"/>
       <c r="B68" s="2" t="n"/>
-      <c r="C68" s="2" t="n"/>
+      <c r="C68" s="2" t="inlineStr"/>
       <c r="D68" s="2" t="n"/>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="E68" s="2" t="n"/>
+      <c r="F68" s="2" t="n"/>
+      <c r="G68" s="2" t="inlineStr">
         <is>
           <t>3.4.3</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr">
+      <c r="H68" s="2" t="inlineStr">
         <is>
           <t>Major industrial complex</t>
         </is>
       </c>
+      <c r="I68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n"/>
       <c r="B69" s="2" t="n"/>
-      <c r="C69" s="2" t="n"/>
+      <c r="C69" s="2" t="inlineStr"/>
       <c r="D69" s="2" t="n"/>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="E69" s="2" t="n"/>
+      <c r="F69" s="2" t="n"/>
+      <c r="G69" s="2" t="inlineStr">
         <is>
           <t>3.4.4</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr">
+      <c r="H69" s="2" t="inlineStr">
         <is>
           <t>Sawmill</t>
         </is>
       </c>
+      <c r="I69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n"/>
       <c r="B70" s="2" t="n"/>
-      <c r="C70" s="2" t="n"/>
+      <c r="C70" s="2" t="inlineStr"/>
       <c r="D70" s="2" t="n"/>
-      <c r="E70" s="2" t="inlineStr">
+      <c r="E70" s="2" t="n"/>
+      <c r="F70" s="2" t="n"/>
+      <c r="G70" s="2" t="inlineStr">
         <is>
           <t>3.4.5</t>
         </is>
       </c>
-      <c r="F70" s="2" t="inlineStr">
+      <c r="H70" s="2" t="inlineStr">
         <is>
           <t>Farm buildings/infrastructure</t>
         </is>
       </c>
+      <c r="I70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n"/>
       <c r="B71" s="2" t="n"/>
-      <c r="C71" s="2" t="n"/>
+      <c r="C71" s="2" t="inlineStr"/>
       <c r="D71" s="2" t="n"/>
-      <c r="E71" s="2" t="inlineStr">
+      <c r="E71" s="2" t="n"/>
+      <c r="F71" s="2" t="n"/>
+      <c r="G71" s="2" t="inlineStr">
         <is>
           <t>3.4.6</t>
         </is>
       </c>
-      <c r="F71" s="2" t="inlineStr">
+      <c r="H71" s="2" t="inlineStr">
         <is>
           <t>Abattoirs</t>
         </is>
       </c>
+      <c r="I71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n"/>
       <c r="B72" s="2" t="n"/>
-      <c r="C72" s="2" t="inlineStr">
+      <c r="C72" s="2" t="inlineStr"/>
+      <c r="D72" s="2" t="inlineStr">
         <is>
           <t>3.5.0</t>
         </is>
       </c>
-      <c r="D72" s="2" t="inlineStr">
+      <c r="E72" s="2" t="inlineStr">
         <is>
           <t>Utilities</t>
         </is>
       </c>
-      <c r="E72" s="2" t="inlineStr">
+      <c r="F72" s="26" t="inlineStr">
+        <is>
+          <t>#F8ADFA</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
         <is>
           <t>3.5.1</t>
         </is>
       </c>
-      <c r="F72" s="2" t="inlineStr">
+      <c r="H72" s="2" t="inlineStr">
         <is>
           <t>Fuel powered electricity generation</t>
         </is>
       </c>
+      <c r="I72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n"/>
       <c r="B73" s="2" t="n"/>
-      <c r="C73" s="2" t="n"/>
+      <c r="C73" s="2" t="inlineStr"/>
       <c r="D73" s="2" t="n"/>
-      <c r="E73" s="2" t="inlineStr">
+      <c r="E73" s="2" t="n"/>
+      <c r="F73" s="2" t="n"/>
+      <c r="G73" s="2" t="inlineStr">
         <is>
           <t>3.5.2</t>
         </is>
       </c>
-      <c r="F73" s="2" t="inlineStr">
+      <c r="H73" s="2" t="inlineStr">
         <is>
           <t>Hydroelectricity generation</t>
         </is>
       </c>
+      <c r="I73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n"/>
       <c r="B74" s="2" t="n"/>
-      <c r="C74" s="2" t="n"/>
+      <c r="C74" s="2" t="inlineStr"/>
       <c r="D74" s="2" t="n"/>
-      <c r="E74" s="2" t="inlineStr">
+      <c r="E74" s="2" t="n"/>
+      <c r="F74" s="2" t="n"/>
+      <c r="G74" s="2" t="inlineStr">
         <is>
           <t>3.5.3</t>
         </is>
       </c>
-      <c r="F74" s="2" t="inlineStr">
+      <c r="H74" s="2" t="inlineStr">
         <is>
           <t>Wind electricity generation</t>
         </is>
       </c>
+      <c r="I74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n"/>
       <c r="B75" s="2" t="n"/>
-      <c r="C75" s="2" t="n"/>
+      <c r="C75" s="2" t="inlineStr"/>
       <c r="D75" s="2" t="n"/>
-      <c r="E75" s="2" t="inlineStr">
+      <c r="E75" s="2" t="n"/>
+      <c r="F75" s="2" t="n"/>
+      <c r="G75" s="2" t="inlineStr">
         <is>
           <t>3.5.4</t>
         </is>
       </c>
-      <c r="F75" s="2" t="inlineStr">
+      <c r="H75" s="2" t="inlineStr">
         <is>
           <t>Solar electricity generation</t>
         </is>
       </c>
+      <c r="I75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n"/>
       <c r="B76" s="2" t="n"/>
-      <c r="C76" s="2" t="n"/>
+      <c r="C76" s="2" t="inlineStr"/>
       <c r="D76" s="2" t="n"/>
-      <c r="E76" s="2" t="inlineStr">
+      <c r="E76" s="2" t="n"/>
+      <c r="F76" s="2" t="n"/>
+      <c r="G76" s="2" t="inlineStr">
         <is>
           <t>3.5.5</t>
         </is>
       </c>
-      <c r="F76" s="2" t="inlineStr">
+      <c r="H76" s="2" t="inlineStr">
         <is>
           <t>Electricity substations and transmission</t>
         </is>
       </c>
+      <c r="I76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n"/>
       <c r="B77" s="2" t="n"/>
-      <c r="C77" s="2" t="n"/>
+      <c r="C77" s="2" t="inlineStr"/>
       <c r="D77" s="2" t="n"/>
-      <c r="E77" s="2" t="inlineStr">
+      <c r="E77" s="2" t="n"/>
+      <c r="F77" s="2" t="n"/>
+      <c r="G77" s="2" t="inlineStr">
         <is>
           <t>3.5.6</t>
         </is>
       </c>
-      <c r="F77" s="2" t="inlineStr">
+      <c r="H77" s="2" t="inlineStr">
         <is>
           <t>Gas treatment, storage, and transmission</t>
         </is>
       </c>
+      <c r="I77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n"/>
       <c r="B78" s="2" t="n"/>
-      <c r="C78" s="2" t="n"/>
+      <c r="C78" s="2" t="inlineStr"/>
       <c r="D78" s="2" t="n"/>
-      <c r="E78" s="2" t="inlineStr">
+      <c r="E78" s="2" t="n"/>
+      <c r="F78" s="2" t="n"/>
+      <c r="G78" s="2" t="inlineStr">
         <is>
           <t>3.5.7</t>
         </is>
       </c>
-      <c r="F78" s="2" t="inlineStr">
+      <c r="H78" s="2" t="inlineStr">
         <is>
           <t>Water extraction and transmission</t>
         </is>
       </c>
+      <c r="I78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n"/>
       <c r="B79" s="2" t="n"/>
-      <c r="C79" s="2" t="inlineStr">
+      <c r="C79" s="2" t="inlineStr"/>
+      <c r="D79" s="2" t="inlineStr">
         <is>
           <t>3.6.0</t>
         </is>
       </c>
-      <c r="D79" s="2" t="inlineStr">
+      <c r="E79" s="2" t="inlineStr">
         <is>
           <t>Transport and communication</t>
         </is>
       </c>
-      <c r="E79" s="2" t="inlineStr">
+      <c r="F79" s="27" t="inlineStr">
+        <is>
+          <t>#72737E</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
         <is>
           <t>3.6.1</t>
         </is>
       </c>
-      <c r="F79" s="2" t="inlineStr">
+      <c r="H79" s="2" t="inlineStr">
         <is>
           <t>Airports/aerodromes</t>
         </is>
       </c>
+      <c r="I79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n"/>
       <c r="B80" s="2" t="n"/>
-      <c r="C80" s="2" t="n"/>
+      <c r="C80" s="2" t="inlineStr"/>
       <c r="D80" s="2" t="n"/>
-      <c r="E80" s="2" t="inlineStr">
+      <c r="E80" s="2" t="n"/>
+      <c r="F80" s="2" t="n"/>
+      <c r="G80" s="2" t="inlineStr">
         <is>
           <t>3.6.2</t>
         </is>
       </c>
-      <c r="F80" s="2" t="inlineStr">
+      <c r="H80" s="2" t="inlineStr">
         <is>
           <t>Roads</t>
         </is>
       </c>
+      <c r="I80" s="2" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n"/>
       <c r="B81" s="2" t="n"/>
-      <c r="C81" s="2" t="n"/>
+      <c r="C81" s="2" t="inlineStr"/>
       <c r="D81" s="2" t="n"/>
-      <c r="E81" s="2" t="inlineStr">
+      <c r="E81" s="2" t="n"/>
+      <c r="F81" s="2" t="n"/>
+      <c r="G81" s="2" t="inlineStr">
         <is>
           <t>3.6.3</t>
         </is>
       </c>
-      <c r="F81" s="2" t="inlineStr">
+      <c r="H81" s="2" t="inlineStr">
         <is>
           <t>Railways</t>
         </is>
       </c>
+      <c r="I81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n"/>
       <c r="B82" s="2" t="n"/>
-      <c r="C82" s="2" t="n"/>
+      <c r="C82" s="2" t="inlineStr"/>
       <c r="D82" s="2" t="n"/>
-      <c r="E82" s="2" t="inlineStr">
+      <c r="E82" s="2" t="n"/>
+      <c r="F82" s="2" t="n"/>
+      <c r="G82" s="2" t="inlineStr">
         <is>
           <t>3.6.4</t>
         </is>
       </c>
-      <c r="F82" s="2" t="inlineStr">
+      <c r="H82" s="2" t="inlineStr">
         <is>
           <t>Ports and water transport</t>
         </is>
       </c>
+      <c r="I82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n"/>
       <c r="B83" s="2" t="n"/>
-      <c r="C83" s="2" t="n"/>
+      <c r="C83" s="2" t="inlineStr"/>
       <c r="D83" s="2" t="n"/>
-      <c r="E83" s="2" t="inlineStr">
+      <c r="E83" s="2" t="n"/>
+      <c r="F83" s="2" t="n"/>
+      <c r="G83" s="2" t="inlineStr">
         <is>
           <t>3.6.5</t>
         </is>
       </c>
-      <c r="F83" s="2" t="inlineStr">
+      <c r="H83" s="2" t="inlineStr">
         <is>
           <t>Navigation and communication</t>
         </is>
       </c>
+      <c r="I83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n"/>
       <c r="B84" s="2" t="n"/>
-      <c r="C84" s="2" t="inlineStr">
+      <c r="C84" s="2" t="inlineStr"/>
+      <c r="D84" s="2" t="inlineStr">
         <is>
           <t>3.7.0</t>
         </is>
       </c>
-      <c r="D84" s="2" t="inlineStr">
+      <c r="E84" s="2" t="inlineStr">
         <is>
           <t>Mining</t>
         </is>
       </c>
-      <c r="E84" s="2" t="inlineStr">
+      <c r="F84" s="28" t="inlineStr">
+        <is>
+          <t>#E1CEA7</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
         <is>
           <t>3.7.1</t>
         </is>
       </c>
-      <c r="F84" s="2" t="inlineStr">
+      <c r="H84" s="2" t="inlineStr">
         <is>
           <t>Mines</t>
         </is>
       </c>
+      <c r="I84" s="2" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n"/>
       <c r="B85" s="2" t="n"/>
-      <c r="C85" s="2" t="n"/>
+      <c r="C85" s="2" t="inlineStr"/>
       <c r="D85" s="2" t="n"/>
-      <c r="E85" s="2" t="inlineStr">
+      <c r="E85" s="2" t="n"/>
+      <c r="F85" s="2" t="n"/>
+      <c r="G85" s="2" t="inlineStr">
         <is>
           <t>3.7.2</t>
         </is>
       </c>
-      <c r="F85" s="2" t="inlineStr">
+      <c r="H85" s="2" t="inlineStr">
         <is>
           <t>Quarries</t>
         </is>
       </c>
+      <c r="I85" s="2" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n"/>
       <c r="B86" s="2" t="n"/>
-      <c r="C86" s="2" t="n"/>
+      <c r="C86" s="2" t="inlineStr"/>
       <c r="D86" s="2" t="n"/>
-      <c r="E86" s="2" t="inlineStr">
+      <c r="E86" s="2" t="n"/>
+      <c r="F86" s="2" t="n"/>
+      <c r="G86" s="2" t="inlineStr">
         <is>
           <t>3.7.3</t>
         </is>
       </c>
-      <c r="F86" s="2" t="inlineStr">
+      <c r="H86" s="2" t="inlineStr">
         <is>
           <t>Tailings</t>
         </is>
       </c>
+      <c r="I86" s="2" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n"/>
       <c r="B87" s="2" t="n"/>
-      <c r="C87" s="2" t="n"/>
+      <c r="C87" s="2" t="inlineStr"/>
       <c r="D87" s="2" t="n"/>
-      <c r="E87" s="2" t="inlineStr">
+      <c r="E87" s="2" t="n"/>
+      <c r="F87" s="2" t="n"/>
+      <c r="G87" s="2" t="inlineStr">
         <is>
           <t>3.7.4</t>
         </is>
       </c>
-      <c r="F87" s="2" t="inlineStr">
+      <c r="H87" s="2" t="inlineStr">
         <is>
           <t>Evaporation basins</t>
         </is>
       </c>
+      <c r="I87" s="2" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n"/>
       <c r="B88" s="2" t="n"/>
-      <c r="C88" s="2" t="n"/>
+      <c r="C88" s="2" t="inlineStr"/>
       <c r="D88" s="2" t="n"/>
-      <c r="E88" s="2" t="inlineStr">
+      <c r="E88" s="2" t="n"/>
+      <c r="F88" s="2" t="n"/>
+      <c r="G88" s="2" t="inlineStr">
         <is>
           <t>3.7.5</t>
         </is>
       </c>
-      <c r="F88" s="2" t="inlineStr">
+      <c r="H88" s="2" t="inlineStr">
         <is>
           <t>Extractive industry not in use</t>
         </is>
       </c>
+      <c r="I88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n"/>
       <c r="B89" s="2" t="n"/>
-      <c r="C89" s="2" t="inlineStr">
+      <c r="C89" s="2" t="inlineStr"/>
+      <c r="D89" s="2" t="inlineStr">
         <is>
           <t>3.8.0</t>
         </is>
       </c>
-      <c r="D89" s="2" t="inlineStr">
+      <c r="E89" s="2" t="inlineStr">
         <is>
           <t>Waste treatment and disposal</t>
         </is>
       </c>
-      <c r="E89" s="2" t="inlineStr">
+      <c r="F89" s="29" t="inlineStr">
+        <is>
+          <t>#E77148</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
         <is>
           <t>3.8.1</t>
         </is>
       </c>
-      <c r="F89" s="2" t="inlineStr">
+      <c r="H89" s="2" t="inlineStr">
         <is>
           <t>Landfills</t>
         </is>
       </c>
+      <c r="I89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n"/>
       <c r="B90" s="2" t="n"/>
-      <c r="C90" s="2" t="n"/>
+      <c r="C90" s="2" t="inlineStr"/>
       <c r="D90" s="2" t="n"/>
-      <c r="E90" s="2" t="inlineStr">
+      <c r="E90" s="2" t="n"/>
+      <c r="F90" s="2" t="n"/>
+      <c r="G90" s="2" t="inlineStr">
         <is>
           <t>3.8.2</t>
         </is>
       </c>
-      <c r="F90" s="2" t="inlineStr">
+      <c r="H90" s="2" t="inlineStr">
         <is>
           <t>Transfer stations and recycling facilities</t>
         </is>
       </c>
+      <c r="I90" s="2" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n"/>
       <c r="B91" s="2" t="n"/>
-      <c r="C91" s="2" t="n"/>
+      <c r="C91" s="2" t="inlineStr"/>
       <c r="D91" s="2" t="n"/>
-      <c r="E91" s="2" t="inlineStr">
+      <c r="E91" s="2" t="n"/>
+      <c r="F91" s="2" t="n"/>
+      <c r="G91" s="2" t="inlineStr">
         <is>
           <t>3.8.3</t>
         </is>
       </c>
-      <c r="F91" s="2" t="inlineStr">
+      <c r="H91" s="2" t="inlineStr">
         <is>
           <t>Municipal wastewater</t>
         </is>
       </c>
+      <c r="I91" s="2" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n"/>
       <c r="B92" s="2" t="n"/>
-      <c r="C92" s="2" t="n"/>
+      <c r="C92" s="2" t="inlineStr"/>
       <c r="D92" s="2" t="n"/>
-      <c r="E92" s="2" t="inlineStr">
+      <c r="E92" s="2" t="n"/>
+      <c r="F92" s="2" t="n"/>
+      <c r="G92" s="2" t="inlineStr">
         <is>
           <t>3.8.4</t>
         </is>
       </c>
-      <c r="F92" s="2" t="inlineStr">
+      <c r="H92" s="2" t="inlineStr">
         <is>
           <t>Wastewater treatment – land application</t>
         </is>
       </c>
+      <c r="I92" s="2" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n"/>
       <c r="B93" s="2" t="n"/>
-      <c r="C93" s="2" t="n"/>
+      <c r="C93" s="2" t="inlineStr"/>
       <c r="D93" s="2" t="n"/>
-      <c r="E93" s="2" t="inlineStr">
+      <c r="E93" s="2" t="n"/>
+      <c r="F93" s="2" t="n"/>
+      <c r="G93" s="2" t="inlineStr">
         <is>
           <t>3.8.5</t>
         </is>
       </c>
-      <c r="F93" s="2" t="inlineStr">
+      <c r="H93" s="2" t="inlineStr">
         <is>
           <t>Stormwater management</t>
         </is>
       </c>
+      <c r="I93" s="2" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n"/>
       <c r="B94" s="2" t="n"/>
-      <c r="C94" s="2" t="inlineStr">
+      <c r="C94" s="2" t="inlineStr"/>
+      <c r="D94" s="2" t="inlineStr">
         <is>
           <t>3.9.0</t>
         </is>
       </c>
-      <c r="D94" s="2" t="inlineStr">
+      <c r="E94" s="2" t="inlineStr">
         <is>
           <t>Vacant and transitioning land</t>
         </is>
       </c>
-      <c r="E94" s="2" t="inlineStr">
+      <c r="F94" s="30" t="inlineStr">
+        <is>
+          <t>#D69B97</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
         <is>
           <t>3.9.1</t>
         </is>
       </c>
-      <c r="F94" s="2" t="inlineStr">
+      <c r="H94" s="2" t="inlineStr">
         <is>
           <t>Vacant land</t>
         </is>
       </c>
+      <c r="I94" s="2" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n"/>
       <c r="B95" s="2" t="n"/>
-      <c r="C95" s="2" t="n"/>
+      <c r="C95" s="2" t="inlineStr"/>
       <c r="D95" s="2" t="n"/>
-      <c r="E95" s="2" t="inlineStr">
+      <c r="E95" s="2" t="n"/>
+      <c r="F95" s="2" t="n"/>
+      <c r="G95" s="2" t="inlineStr">
         <is>
           <t>3.9.2</t>
         </is>
       </c>
-      <c r="F95" s="2" t="inlineStr">
+      <c r="H95" s="2" t="inlineStr">
         <is>
           <t>Greenfield development</t>
         </is>
       </c>
+      <c r="I95" s="2" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n"/>
       <c r="B96" s="2" t="n"/>
-      <c r="C96" s="2" t="n"/>
+      <c r="C96" s="2" t="inlineStr"/>
       <c r="D96" s="2" t="n"/>
-      <c r="E96" s="2" t="inlineStr">
+      <c r="E96" s="2" t="n"/>
+      <c r="F96" s="2" t="n"/>
+      <c r="G96" s="2" t="inlineStr">
         <is>
           <t>3.9.3</t>
         </is>
       </c>
-      <c r="F96" s="2" t="inlineStr">
+      <c r="H96" s="2" t="inlineStr">
         <is>
           <t>Brownfield development</t>
         </is>
       </c>
+      <c r="I96" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="48">
-    <mergeCell ref="C27:C29"/>
-    <mergeCell ref="C57:C59"/>
+  <mergeCells count="68">
+    <mergeCell ref="A2:A21"/>
+    <mergeCell ref="A22:A52"/>
+    <mergeCell ref="A53:A96"/>
+    <mergeCell ref="B2:B21"/>
+    <mergeCell ref="B22:B52"/>
+    <mergeCell ref="B53:B96"/>
+    <mergeCell ref="D2:D8"/>
+    <mergeCell ref="D9:D11"/>
+    <mergeCell ref="D12:D19"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="D22:D26"/>
+    <mergeCell ref="D27:D29"/>
+    <mergeCell ref="D30:D33"/>
+    <mergeCell ref="D34:D36"/>
+    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="D39:D43"/>
+    <mergeCell ref="D44:D48"/>
+    <mergeCell ref="D49:D52"/>
+    <mergeCell ref="D53:D56"/>
+    <mergeCell ref="D57:D59"/>
     <mergeCell ref="D60:D65"/>
-    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D66:D71"/>
     <mergeCell ref="D72:D78"/>
-    <mergeCell ref="C2:C8"/>
-    <mergeCell ref="C30:C33"/>
-    <mergeCell ref="D49:D52"/>
-    <mergeCell ref="C39:C43"/>
-    <mergeCell ref="D9:D11"/>
-    <mergeCell ref="C22:C26"/>
-    <mergeCell ref="D39:D43"/>
-    <mergeCell ref="A2:A21"/>
-    <mergeCell ref="C34:C36"/>
     <mergeCell ref="D79:D83"/>
-    <mergeCell ref="C72:C78"/>
+    <mergeCell ref="D84:D88"/>
     <mergeCell ref="D89:D93"/>
     <mergeCell ref="D94:D96"/>
-    <mergeCell ref="B53:B96"/>
-    <mergeCell ref="A22:A52"/>
-    <mergeCell ref="D44:D48"/>
-    <mergeCell ref="D66:D71"/>
-    <mergeCell ref="D22:D26"/>
-    <mergeCell ref="D84:D88"/>
-    <mergeCell ref="D34:D36"/>
-    <mergeCell ref="A53:A96"/>
-    <mergeCell ref="C12:C19"/>
-    <mergeCell ref="D37:D38"/>
-    <mergeCell ref="C89:C93"/>
-    <mergeCell ref="C94:C96"/>
-    <mergeCell ref="D30:D33"/>
-    <mergeCell ref="D53:D56"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="D27:D29"/>
-    <mergeCell ref="C79:C83"/>
-    <mergeCell ref="B22:B52"/>
-    <mergeCell ref="C44:C48"/>
-    <mergeCell ref="C60:C65"/>
-    <mergeCell ref="C66:C71"/>
-    <mergeCell ref="D12:D19"/>
-    <mergeCell ref="D57:D59"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="C84:C88"/>
-    <mergeCell ref="D2:D8"/>
-    <mergeCell ref="C53:C56"/>
-    <mergeCell ref="B2:B21"/>
-    <mergeCell ref="C9:C11"/>
-    <mergeCell ref="C49:C52"/>
+    <mergeCell ref="E2:E8"/>
+    <mergeCell ref="E9:E11"/>
+    <mergeCell ref="E12:E19"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="E22:E26"/>
+    <mergeCell ref="E27:E29"/>
+    <mergeCell ref="E30:E33"/>
+    <mergeCell ref="E34:E36"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="E39:E43"/>
+    <mergeCell ref="E44:E48"/>
+    <mergeCell ref="E49:E52"/>
+    <mergeCell ref="E53:E56"/>
+    <mergeCell ref="E57:E59"/>
+    <mergeCell ref="E60:E65"/>
+    <mergeCell ref="E66:E71"/>
+    <mergeCell ref="E72:E78"/>
+    <mergeCell ref="E79:E83"/>
+    <mergeCell ref="E84:E88"/>
+    <mergeCell ref="E89:E93"/>
+    <mergeCell ref="E94:E96"/>
+    <mergeCell ref="F9:F11"/>
+    <mergeCell ref="F12:F19"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="F22:F26"/>
+    <mergeCell ref="F27:F29"/>
+    <mergeCell ref="F30:F33"/>
+    <mergeCell ref="F34:F36"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="F39:F43"/>
+    <mergeCell ref="F44:F48"/>
+    <mergeCell ref="F49:F52"/>
+    <mergeCell ref="F53:F56"/>
+    <mergeCell ref="F57:F59"/>
+    <mergeCell ref="F60:F65"/>
+    <mergeCell ref="F66:F71"/>
+    <mergeCell ref="F72:F78"/>
+    <mergeCell ref="F79:F83"/>
+    <mergeCell ref="F84:F88"/>
+    <mergeCell ref="F89:F93"/>
+    <mergeCell ref="F94:F96"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>